<commit_message>
Preserve inherited stage three growth implementation draft
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/game_rules.xlsx
+++ b/space-battleship/config_excel/game_rules.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="game_rules" sheetId="1" r:id="Rf0ab8a2970774fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="game_rules" sheetId="1" r:id="Ra80ab035dfb44841"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -428,6 +428,94 @@
         <x:v>Existing native reactive armour: damage reduction per stack.</x:v>
       </x:c>
     </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="1" t="str">
+        <x:v>research_ai_divisor</x:v>
+      </x:c>
+      <x:c r="B15" s="1" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C15" s="1" t="str">
+        <x:v>Design 03: base AI work speed divisor; initial one AI gives speed one.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="1" t="str">
+        <x:v>research_invest_log_divisor</x:v>
+      </x:c>
+      <x:c r="B16" s="1" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C16" s="1" t="str">
+        <x:v>Design 03: investment work multiplier is 1+log10(rate)/divisor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="1" t="str">
+        <x:v>research_peak_log_divisor</x:v>
+      </x:c>
+      <x:c r="B17" s="1" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="C17" s="1" t="str">
+        <x:v>Design 03: unification historical peak factor divisor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="1" t="str">
+        <x:v>research_income_window</x:v>
+      </x:c>
+      <x:c r="B18" s="1" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Design 01/03: income windows and automatic investment refresh, game/wall seconds.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="1" t="str">
+        <x:v>research_minimum_ratio</x:v>
+      </x:c>
+      <x:c r="B19" s="1" t="n">
+        <x:v>0.001</x:v>
+      </x:c>
+      <x:c r="C19" s="1" t="str">
+        <x:v>Design 01: minimum automatic investment fraction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="1" t="str">
+        <x:v>research_default_ratio</x:v>
+      </x:c>
+      <x:c r="B20" s="1" t="n">
+        <x:v>0.01</x:v>
+      </x:c>
+      <x:c r="C20" s="1" t="str">
+        <x:v>Design 01: initial automatic investment fraction.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="1" t="str">
+        <x:v>hyperspace_unlock_reached</x:v>
+      </x:c>
+      <x:c r="B21" s="1" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C21" s="1" t="str">
+        <x:v>Design 01: reached stage gate for evolution material availability.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="1" t="str">
+        <x:v>higgs_minimum_width</x:v>
+      </x:c>
+      <x:c r="B22" s="1" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C22" s="1" t="str">
+        <x:v>Design 02: Higgs full width uses max(this value, rail_trail_width) before its area bonus.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>